<commit_message>
Actualizacion formatos e imagen bomberos
</commit_message>
<xml_diff>
--- a/X/BD.xlsx
+++ b/X/BD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/X/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7755" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{504CB249-8542-4AC9-97FE-FC2FB54E87FD}"/>
+  <xr:revisionPtr revIDLastSave="7756" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A045170-2CF0-4204-A969-92358F342CB1}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>
@@ -11892,10 +11892,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
@@ -12216,6 +12212,7 @@
   <dimension ref="A1:LH200"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="18" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="11.5546875" style="9"/>

</xml_diff>